<commit_message>
Cada oferta por turma com seu Classroom
</commit_message>
<xml_diff>
--- a/public/jobs/ofertas/B4-2026.xlsx
+++ b/public/jobs/ofertas/B4-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Downloads\montador_de_grade_unifil\public\jobs\ofertas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{05A47706-7B6C-4C56-BD1B-11352DA7793C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97F76DF1-B399-45A2-9049-4392C82857CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BB45BF00-CC24-488C-B190-8EDA9BDC1E77}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8551CB66-AFFC-4736-8187-74AC573681ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Aulas" sheetId="1" r:id="rId1"/>
@@ -615,6 +615,9 @@
     <t>Qualidade de Software: Normas, Modelos e Melhoria Contínua</t>
   </si>
   <si>
+    <t>fzbos4xl</t>
+  </si>
+  <si>
     <t>ESDS230005</t>
   </si>
   <si>
@@ -631,9 +634,6 @@
   </si>
   <si>
     <t>l63gjoop</t>
-  </si>
-  <si>
-    <t>fzbos4xl</t>
   </si>
   <si>
     <t>COAP230024</t>
@@ -994,35 +994,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A87FCEAD-C4DC-4395-A50A-63DB3C4B398D}" name="Tabela1" displayName="Tabela1" ref="A1:K217" totalsRowShown="0" headerRowDxfId="7">
-  <autoFilter ref="A1:K217" xr:uid="{A87FCEAD-C4DC-4395-A50A-63DB3C4B398D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E3389BCB-67F4-4121-8B90-9E87C40B3A62}" name="Tabela1" displayName="Tabela1" ref="A1:K217" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:K217" xr:uid="{E3389BCB-67F4-4121-8B90-9E87C40B3A62}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{CF07484D-9F49-4D8A-897E-9131A5389B30}" name="Código" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{37AB9928-2916-4A57-A6AC-E0A120558F4C}" name="Disciplina" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{76239738-0F6F-4779-8D2A-92ED65811A1E}" name="Dia" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{F4999CCB-2E26-4B11-A763-1D8469E1BBF7}" name="Horário" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{7C1CE0F2-548F-4B06-AD5D-BE2C4078531A}" name="Turma" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{415F6232-DA89-4842-A297-A0FE7A3AFD83}" name="Curso" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{11EBF355-6CF9-45C6-9279-0A35C88B8888}" name="Sala" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{DC146632-ECDD-407D-A040-36512076FEDB}" name="Professor" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{35A6B302-127F-4C58-A1D2-73F1283E655E}" name="Tipo" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{EE8CC09D-140D-421D-AB60-044046DCB423}" name="C.H." dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{A510CE5F-4CB0-48C5-9EE3-5559F3D08E00}" name="Classroom" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{8BC8BBE2-2B06-49B6-9BE6-0B3F037651B7}" name="Código" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{90142ACC-34D4-4C08-AD91-88564D786B1F}" name="Disciplina" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{547F7103-83FF-4687-AC03-D343C6F92A96}" name="Dia" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{77D70436-BF81-4392-88E9-636ECC5E21E5}" name="Horário" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{C86778ED-47B4-4E12-8C9B-04D8214A9BD9}" name="Turma" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{BCD10354-8799-4FCE-B520-97068DB086C5}" name="Curso" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{07DDB65A-F2FD-4020-B8F9-66CF85FB27D2}" name="Sala" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{564409E2-DAEE-4ED7-8FDB-CB9E1CBC2583}" name="Professor" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{1FE7DDEC-327A-4DF9-939E-734801CA549A}" name="Tipo" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{00EC796E-7BE6-43D0-9D37-2689A4CC8884}" name="C.H." dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{1FA7A86D-613D-4689-8289-9384643BF11F}" name="Classroom" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4CF00C92-D394-440C-A9A0-609EDD386ACB}" name="Tabela2" displayName="Tabela2" ref="A1:F40" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:F40" xr:uid="{4CF00C92-D394-440C-A9A0-609EDD386ACB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A28EE10D-3AC1-4A80-A3C4-E3DC32496522}" name="Tabela2" displayName="Tabela2" ref="A1:F40" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:F40" xr:uid="{A28EE10D-3AC1-4A80-A3C4-E3DC32496522}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{394D1651-CF9C-4EE8-9354-F50E6C27BC54}" name="Código" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{F9F50181-0BBD-4DCF-AC8A-AC98ADBB72A9}" name="Disciplina" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{90AECA33-1BB9-425F-B89A-66251FD79FD1}" name="Turma" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{01E9C998-048E-49EF-B452-0DC9C7239B7F}" name="Curso" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{B3FC5577-55E3-422C-9DE1-6F2186E265CD}" name="Professor" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{525ABBF5-7F48-4412-B8C5-68B975B78FB3}" name="C.H." dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{26DEAB5D-6500-4DC1-A176-39E600878AB6}" name="Código" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{200061F1-B93A-4C66-A4DC-D49C50830970}" name="Disciplina" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{397C4D51-85FA-447D-BAF0-E2AEDD7D0B69}" name="Turma" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{5E68897C-BE87-4CBF-B88C-F00784966CA2}" name="Curso" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{BC23B21C-CAED-43E5-B9D2-3E5344407BCD}" name="Professor" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{B6749076-0441-41F3-A0B8-0F6063D40EC8}" name="C.H." dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1344,7 +1344,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CAE710A-ACCC-4172-AE55-70414BFEAF03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527B2ED1-9E5C-47FF-84F5-99E37B12D0AA}">
   <dimension ref="A1:K217"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6609,15 +6609,15 @@
         <v>33</v>
       </c>
       <c r="K150" s="1" t="s">
-        <v>20</v>
+        <v>192</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>24</v>
@@ -6644,15 +6644,15 @@
         <v>20</v>
       </c>
       <c r="K151" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>30</v>
@@ -6679,7 +6679,7 @@
         <v>26</v>
       </c>
       <c r="K152" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
@@ -6714,7 +6714,7 @@
         <v>33</v>
       </c>
       <c r="K153" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
@@ -6994,15 +6994,15 @@
         <v>33</v>
       </c>
       <c r="K161" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>24</v>
@@ -7029,7 +7029,7 @@
         <v>20</v>
       </c>
       <c r="K162" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
@@ -7099,7 +7099,7 @@
         <v>33</v>
       </c>
       <c r="K164" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.25">
@@ -8966,7 +8966,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20ADFAC-CD8A-47C5-8434-4A05953D15FE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A7961C-CEF8-4145-8A41-88630852FA7B}">
   <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>